<commit_message>
Added Pi Pico 2s to database
</commit_message>
<xml_diff>
--- a/To Add v2/ICs - Embedded - MCU - Module.xlsx
+++ b/To Add v2/ICs - Embedded - MCU - Module.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\To Add v2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E525C9A-A692-4B0F-96AD-D8038ECB9D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D9E39A-7F9B-4728-A50B-298149E0FC47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="7725" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="49">
   <si>
     <t>Totals</t>
   </si>
@@ -104,9 +104,6 @@
     <t>Arduino Nano Every</t>
   </si>
   <si>
-    <t>Arduino Mega 2560</t>
-  </si>
-  <si>
     <t>Arduino</t>
   </si>
   <si>
@@ -122,15 +119,6 @@
     <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/697/ABX00033_Web.pdf</t>
   </si>
   <si>
-    <t>A000067</t>
-  </si>
-  <si>
-    <t>1050-1018-ND</t>
-  </si>
-  <si>
-    <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/2275/A000067_Web.pdf</t>
-  </si>
-  <si>
     <t> </t>
   </si>
   <si>
@@ -183,6 +171,18 @@
   </si>
   <si>
     <t>MCU_Boards:Pi_Pico_2_SMD</t>
+  </si>
+  <si>
+    <t>Pi Pico 2H</t>
+  </si>
+  <si>
+    <t>SC1632</t>
+  </si>
+  <si>
+    <t>2648-SC1632-ND</t>
+  </si>
+  <si>
+    <t>0Dan_MCUs:Pi_Pico_2</t>
   </si>
 </sst>
 </file>
@@ -528,21 +528,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="17.36328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="B1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -580,25 +581,25 @@
       </c>
       <c r="K2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L2">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T2" t="s">
         <v>1</v>
       </c>
       <c r="U2">
         <f>AVERAGE(Q7:Q9999)</f>
-        <v>87.27272727272728</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="T3" t="s">
         <v>2</v>
       </c>
@@ -607,7 +608,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -649,19 +650,19 @@
       </c>
       <c r="U4">
         <f>SUM(R7:R9999)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="T5" t="s">
         <v>5</v>
       </c>
       <c r="U5">
         <f>COUNTIF(Q7:Q9999,"&lt;100")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>6</v>
       </c>
@@ -705,7 +706,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
@@ -721,28 +722,28 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
         <v>23</v>
       </c>
-      <c r="G7" t="s">
+      <c r="I7" t="s">
         <v>25</v>
       </c>
-      <c r="H7" t="s">
-        <v>24</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>26</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
+        <v>28</v>
+      </c>
+      <c r="L7" t="s">
+        <v>29</v>
+      </c>
+      <c r="M7" t="s">
         <v>27</v>
-      </c>
-      <c r="K7" t="s">
-        <v>32</v>
-      </c>
-      <c r="L7" t="s">
-        <v>33</v>
-      </c>
-      <c r="M7" t="s">
-        <v>31</v>
       </c>
       <c r="P7">
         <f>COUNTBLANK(C7:M7)</f>
@@ -764,7 +765,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2</v>
       </c>
@@ -777,31 +778,31 @@
         <v>Arduino Nano R3</v>
       </c>
       <c r="E8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J8" t="s">
         <v>39</v>
       </c>
-      <c r="F8" t="s">
+      <c r="K8" t="s">
         <v>40</v>
       </c>
-      <c r="G8" t="s">
+      <c r="L8" t="s">
         <v>41</v>
       </c>
-      <c r="H8" t="s">
-        <v>42</v>
-      </c>
-      <c r="I8" t="s">
-        <v>41</v>
-      </c>
-      <c r="J8" t="s">
-        <v>43</v>
-      </c>
-      <c r="K8" t="s">
-        <v>44</v>
-      </c>
-      <c r="L8" t="s">
-        <v>45</v>
-      </c>
       <c r="M8" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="P8">
         <f>COUNTBLANK(C8:M8)</f>
@@ -816,7 +817,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>3</v>
+      </c>
       <c r="C9" t="str">
         <f t="shared" ref="C9:C11" si="1">D9</f>
         <v>Pi Pico 2 TH</v>
@@ -826,40 +830,49 @@
         <v>Pi Pico 2 TH</v>
       </c>
       <c r="E9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" t="s">
         <v>34</v>
       </c>
-      <c r="F9" t="s">
-        <v>36</v>
-      </c>
-      <c r="G9" t="s">
-        <v>37</v>
-      </c>
-      <c r="H9" t="s">
-        <v>24</v>
-      </c>
-      <c r="I9" t="s">
-        <v>38</v>
-      </c>
       <c r="J9" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
+      </c>
+      <c r="K9" t="s">
+        <v>48</v>
       </c>
       <c r="L9" t="s">
-        <v>47</v>
+        <v>43</v>
+      </c>
+      <c r="M9" t="s">
+        <v>27</v>
       </c>
       <c r="P9">
-        <f t="shared" ref="P9:P13" si="3">COUNTBLANK(C9:M9)</f>
-        <v>2</v>
+        <f t="shared" ref="P9:P11" si="3">COUNTBLANK(C9:M9)</f>
+        <v>0</v>
       </c>
       <c r="Q9">
-        <f t="shared" ref="Q9:Q13" si="4">100*COUNTA(C9:M9)/$U$7</f>
-        <v>81.818181818181813</v>
+        <f t="shared" ref="Q9:Q11" si="4">100*COUNTA(C9:M9)/$U$7</f>
+        <v>100</v>
       </c>
       <c r="R9">
-        <f t="shared" ref="R9:R13" si="5">IF(Q9=100,1,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+        <f t="shared" ref="R9:R11" si="5">IF(Q9=100,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>4</v>
+      </c>
       <c r="C10" t="str">
         <f t="shared" si="1"/>
         <v>Pi Pico 2 SMD</v>
@@ -869,77 +882,93 @@
         <v>Pi Pico 2 SMD</v>
       </c>
       <c r="E10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="G10" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="H10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I10" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="J10" t="s">
-        <v>46</v>
+        <v>42</v>
+      </c>
+      <c r="K10" t="s">
+        <v>48</v>
       </c>
       <c r="L10" t="s">
-        <v>48</v>
+        <v>44</v>
+      </c>
+      <c r="M10" t="s">
+        <v>27</v>
       </c>
       <c r="P10">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q10">
         <f t="shared" si="4"/>
-        <v>81.818181818181813</v>
+        <v>100</v>
       </c>
       <c r="R10">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="C11" t="str">
-        <f t="shared" si="1"/>
-        <v>Arduino Mega 2560</v>
-      </c>
-      <c r="D11" t="str">
-        <f t="shared" si="2"/>
-        <v>Arduino Mega 2560</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" t="s">
+        <v>45</v>
       </c>
       <c r="E11" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" t="s">
         <v>23</v>
       </c>
-      <c r="G11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H11" t="s">
-        <v>24</v>
-      </c>
       <c r="I11" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="J11" t="s">
-        <v>30</v>
+        <v>42</v>
+      </c>
+      <c r="K11" t="s">
+        <v>48</v>
+      </c>
+      <c r="L11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M11" t="s">
+        <v>27</v>
       </c>
       <c r="P11">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q11">
         <f t="shared" si="4"/>
-        <v>72.727272727272734</v>
+        <v>100</v>
       </c>
       <c r="R11">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>